<commit_message>
feat: integrate Telegram Mini App with Next.js frontend and FastAPI backend
</commit_message>
<xml_diff>
--- a/_data_list/FF_Master.xlsx
+++ b/_data_list/FF_Master.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Telegram_Project\OrangeFlow_Dev\_data_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C55751C-11A8-462F-B9BD-D145D903BC78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87194FEE-4304-40C6-A51A-151B25E1344C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AK$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AK$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="314">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -710,9 +710,6 @@
     <t>R645040</t>
   </si>
   <si>
-    <t>7017344002631</t>
-  </si>
-  <si>
     <t>Ajmina</t>
   </si>
   <si>
@@ -960,6 +957,30 @@
   </si>
   <si>
     <t>RYZBRB01</t>
+  </si>
+  <si>
+    <t>RYZBRB01SUP01</t>
+  </si>
+  <si>
+    <t>RSDSO0178</t>
+  </si>
+  <si>
+    <t>Md. Rasel Mia</t>
+  </si>
+  <si>
+    <t>Supervisor</t>
+  </si>
+  <si>
+    <t>Abdul Rouf</t>
+  </si>
+  <si>
+    <t>Samsad Begum</t>
+  </si>
+  <si>
+    <t>Chilni, Itna, Kishoreganj</t>
+  </si>
+  <si>
+    <t>Tanvir</t>
   </si>
 </sst>
 </file>
@@ -1018,7 +1039,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1031,14 +1052,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1362,164 +1400,163 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AK42"/>
+  <dimension ref="A1:AK43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="37.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="39.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="38.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="27" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="27.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="28.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="11.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" style="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29" style="13" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" style="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14" style="13" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10" style="14" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="41.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="44.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="35.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="38.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="27" style="13" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="53.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="32.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="33.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="17.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.5703125" style="13" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="21.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="12.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="38" max="16384" width="9.140625" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="P1" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="R1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="S1" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="T1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U1" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="V1" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="W1" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="X1" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y1" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="Z1" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="AA1" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="AB1" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC1" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="AD1" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="AE1" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="AF1" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="AG1" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="AH1" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="AI1" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="AJ1" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="AK1" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="M1" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="R1" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="S1" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="T1" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="U1" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="V1" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="W1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="X1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y1" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="Z1" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="AA1" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="AB1" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="AC1" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="AD1" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="AE1" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="AF1" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="AG1" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="AH1" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="AI1" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="AJ1" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="AK1" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>304</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>34</v>
@@ -1554,6 +1591,7 @@
       <c r="L2" s="2">
         <v>45505</v>
       </c>
+      <c r="M2" s="2"/>
       <c r="N2" s="1" t="s">
         <v>157</v>
       </c>
@@ -1573,9 +1611,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>35</v>
@@ -1610,6 +1648,7 @@
       <c r="L3" s="2">
         <v>44896</v>
       </c>
+      <c r="M3" s="2"/>
       <c r="N3" s="1" t="s">
         <v>157</v>
       </c>
@@ -1629,9 +1668,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>36</v>
@@ -1666,6 +1705,7 @@
       <c r="L4" s="2">
         <v>43132</v>
       </c>
+      <c r="M4" s="2"/>
       <c r="N4" s="1" t="s">
         <v>157</v>
       </c>
@@ -1685,9 +1725,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>37</v>
@@ -1719,6 +1759,7 @@
       <c r="L5" s="2">
         <v>43160</v>
       </c>
+      <c r="M5" s="2"/>
       <c r="N5" s="1" t="s">
         <v>157</v>
       </c>
@@ -1738,9 +1779,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>38</v>
@@ -1772,6 +1813,7 @@
       <c r="L6" s="2">
         <v>43525</v>
       </c>
+      <c r="M6" s="2"/>
       <c r="N6" s="1" t="s">
         <v>157</v>
       </c>
@@ -1791,9 +1833,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>39</v>
@@ -1825,6 +1867,7 @@
       <c r="L7" s="2">
         <v>45840</v>
       </c>
+      <c r="M7" s="2"/>
       <c r="N7" s="1" t="s">
         <v>157</v>
       </c>
@@ -1844,9 +1887,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>40</v>
@@ -1905,7 +1948,7 @@
     </row>
     <row r="9" spans="1:37" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>154</v>
@@ -1953,7 +1996,7 @@
       <c r="Q9" t="s">
         <v>62</v>
       </c>
-      <c r="R9" s="11">
+      <c r="R9" s="8">
         <v>2311030553506</v>
       </c>
       <c r="U9" s="4" t="s">
@@ -2008,9 +2051,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>41</v>
@@ -2042,6 +2085,7 @@
       <c r="L10" s="2">
         <v>45909</v>
       </c>
+      <c r="M10" s="2"/>
       <c r="N10" s="1" t="s">
         <v>157</v>
       </c>
@@ -2061,9 +2105,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>42</v>
@@ -2098,6 +2142,7 @@
       <c r="L11" s="2">
         <v>45873</v>
       </c>
+      <c r="M11" s="2"/>
       <c r="N11" s="1" t="s">
         <v>157</v>
       </c>
@@ -2117,9 +2162,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>43</v>
@@ -2151,6 +2196,7 @@
       <c r="L12" s="2">
         <v>45976</v>
       </c>
+      <c r="M12" s="2"/>
       <c r="N12" s="1" t="s">
         <v>157</v>
       </c>
@@ -2170,9 +2216,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>44</v>
@@ -2207,6 +2253,7 @@
       <c r="L13" s="2">
         <v>45909</v>
       </c>
+      <c r="M13" s="2"/>
       <c r="N13" s="1" t="s">
         <v>157</v>
       </c>
@@ -2226,9 +2273,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>45</v>
@@ -2260,6 +2307,7 @@
       <c r="L14" s="2">
         <v>45965</v>
       </c>
+      <c r="M14" s="2"/>
       <c r="N14" s="1" t="s">
         <v>157</v>
       </c>
@@ -2279,9 +2327,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>46</v>
@@ -2316,6 +2364,7 @@
       <c r="L15" s="2">
         <v>45748</v>
       </c>
+      <c r="M15" s="2"/>
       <c r="N15" s="1" t="s">
         <v>157</v>
       </c>
@@ -2335,9 +2384,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>47</v>
@@ -2372,6 +2421,7 @@
       <c r="L16" s="2">
         <v>45999</v>
       </c>
+      <c r="M16" s="2"/>
       <c r="N16" s="1" t="s">
         <v>157</v>
       </c>
@@ -2391,9 +2441,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>48</v>
@@ -2428,6 +2478,7 @@
       <c r="L17" s="2">
         <v>43709</v>
       </c>
+      <c r="M17" s="2"/>
       <c r="N17" s="1" t="s">
         <v>157</v>
       </c>
@@ -2447,9 +2498,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>49</v>
@@ -2484,6 +2535,7 @@
       <c r="L18" s="2">
         <v>44470</v>
       </c>
+      <c r="M18" s="2"/>
       <c r="N18" s="1" t="s">
         <v>157</v>
       </c>
@@ -2503,9 +2555,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>50</v>
@@ -2537,6 +2589,7 @@
       <c r="L19" s="2">
         <v>45444</v>
       </c>
+      <c r="M19" s="2"/>
       <c r="N19" s="1" t="s">
         <v>157</v>
       </c>
@@ -2556,9 +2609,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="20" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>51</v>
@@ -2593,6 +2646,7 @@
       <c r="L20" s="2">
         <v>46023</v>
       </c>
+      <c r="M20" s="2"/>
       <c r="N20" s="1" t="s">
         <v>157</v>
       </c>
@@ -2612,9 +2666,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>133</v>
@@ -2640,6 +2694,7 @@
       <c r="L21" s="2">
         <v>42370</v>
       </c>
+      <c r="M21" s="2"/>
       <c r="N21" s="1" t="s">
         <v>157</v>
       </c>
@@ -2656,9 +2711,9 @@
         <v>1731510105407</v>
       </c>
     </row>
-    <row r="22" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>132</v>
@@ -2684,6 +2739,7 @@
       <c r="L22" s="2">
         <v>41122</v>
       </c>
+      <c r="M22" s="2"/>
       <c r="N22" s="1" t="s">
         <v>157</v>
       </c>
@@ -2700,9 +2756,9 @@
         <v>1471030170630</v>
       </c>
     </row>
-    <row r="23" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>130</v>
@@ -2728,6 +2784,7 @@
       <c r="L23" s="2">
         <v>45870</v>
       </c>
+      <c r="M23" s="2"/>
       <c r="N23" s="1" t="s">
         <v>157</v>
       </c>
@@ -2744,9 +2801,9 @@
         <v>1731030011382</v>
       </c>
     </row>
-    <row r="24" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>129</v>
@@ -2772,6 +2829,7 @@
       <c r="L24" s="2">
         <v>46054</v>
       </c>
+      <c r="M24" s="2"/>
       <c r="N24" s="1" t="s">
         <v>157</v>
       </c>
@@ -2789,1298 +2847,1393 @@
       </c>
     </row>
     <row r="25" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B25" s="1" t="s">
+      <c r="A25" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B25" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25" s="13">
         <v>1786080093</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="13">
         <v>1410678746</v>
       </c>
-      <c r="I25" s="1" t="s">
+      <c r="I25" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="13">
         <v>10000</v>
       </c>
-      <c r="L25" s="1">
+      <c r="L25" s="14">
         <v>46082</v>
       </c>
-      <c r="N25" s="1" t="s">
+      <c r="N25" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="O25" s="1">
+      <c r="O25" s="14">
         <v>33834</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="15">
         <v>6404733260</v>
       </c>
-      <c r="Q25" s="1" t="s">
+      <c r="Q25" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="R25" s="1">
+      <c r="R25" s="15">
         <v>1731580493357</v>
       </c>
-      <c r="V25" s="1" t="s">
+      <c r="V25" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="W25" s="1">
+      <c r="W25" s="13">
         <v>1752787879</v>
       </c>
-      <c r="X25" s="1" t="s">
+      <c r="X25" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="Z25" s="1" t="s">
+      <c r="Z25" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="AA25" s="1" t="s">
+      <c r="AA25" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="AB25" s="1" t="s">
+      <c r="AB25" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="AC25" s="1" t="s">
+      <c r="AC25" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="AD25" s="1" t="s">
+      <c r="AD25" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="AE25" s="1" t="s">
+      <c r="AE25" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="AF25" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG25" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH25" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI25" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ25" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK25" s="1" t="s">
+      <c r="AF25" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG25" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH25" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI25" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ25" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK25" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B26" s="1" t="s">
+      <c r="A26" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G26" s="13">
         <v>1410071973</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="13">
         <v>1410071973</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="I26" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="13">
         <v>10000</v>
       </c>
-      <c r="L26" s="1">
+      <c r="L26" s="14">
         <v>46082</v>
       </c>
-      <c r="N26" s="1" t="s">
+      <c r="N26" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="O26" s="1">
+      <c r="O26" s="14">
         <v>32540</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="15">
         <v>1314935507162</v>
       </c>
-      <c r="Q26" s="1" t="s">
+      <c r="Q26" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="R26" s="1">
+      <c r="R26" s="15">
         <v>1731580492738</v>
       </c>
-      <c r="S26" s="1" t="s">
+      <c r="S26" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="V26" s="1" t="s">
+      <c r="V26" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="W26" s="1">
+      <c r="W26" s="13">
         <v>1864929394</v>
       </c>
-      <c r="X26" s="1" t="s">
+      <c r="X26" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="Z26" s="1" t="s">
+      <c r="Z26" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="AA26" s="1" t="s">
+      <c r="AA26" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="AB26" s="1" t="s">
+      <c r="AB26" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="AC26" s="1" t="s">
+      <c r="AC26" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="AD26" s="1" t="s">
+      <c r="AD26" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="AE26" s="1" t="s">
+      <c r="AE26" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="AF26" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG26" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH26" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI26" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ26" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK26" s="1" t="s">
+      <c r="AF26" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG26" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH26" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI26" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ26" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK26" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B27" s="1" t="s">
+      <c r="A27" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B27" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="G27" s="1">
+      <c r="G27" s="13">
         <v>1410240211</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="13">
         <v>1410240211</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="I27" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="13">
         <v>10000</v>
       </c>
-      <c r="L27" s="1">
+      <c r="L27" s="14">
         <v>45971</v>
       </c>
-      <c r="N27" s="1" t="s">
+      <c r="N27" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="O27" s="1">
+      <c r="O27" s="14">
         <v>1</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="15">
         <v>2863545949</v>
       </c>
-      <c r="Q27" s="1" t="s">
+      <c r="Q27" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="R27" s="1">
+      <c r="R27" s="15">
         <v>1731050292189</v>
       </c>
-      <c r="V27" s="1" t="s">
+      <c r="V27" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="W27" s="1">
+      <c r="W27" s="13">
         <v>1407911493</v>
       </c>
-      <c r="X27" s="1" t="s">
+      <c r="X27" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="Z27" s="1" t="s">
+      <c r="Z27" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="AA27" s="1" t="s">
+      <c r="AA27" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="AB27" s="1" t="s">
+      <c r="AB27" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="AC27" s="1" t="s">
+      <c r="AC27" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="AD27" s="1" t="s">
+      <c r="AD27" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="AE27" s="1" t="s">
+      <c r="AE27" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="AF27" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG27" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH27" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI27" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ27" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK27" s="1" t="s">
+      <c r="AF27" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG27" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH27" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI27" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ27" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK27" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B28" s="1" t="s">
+      <c r="A28" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E28" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="G28" s="1">
+      <c r="G28" s="13">
         <v>1917787990</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="13">
         <v>1410436602</v>
       </c>
-      <c r="I28" s="1" t="s">
+      <c r="I28" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="13">
         <v>10000</v>
       </c>
-      <c r="L28" s="1">
+      <c r="L28" s="14">
         <v>45971</v>
       </c>
-      <c r="N28" s="1" t="s">
+      <c r="N28" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="O28" s="1">
+      <c r="O28" s="14">
         <v>31595</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="15">
         <v>4813347971938</v>
       </c>
-      <c r="Q28" s="1" t="s">
+      <c r="Q28" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="R28" s="1">
+      <c r="R28" s="15">
         <v>2311580489016</v>
       </c>
-      <c r="V28" s="1" t="s">
+      <c r="V28" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="W28" s="1">
+      <c r="W28" s="13">
         <v>1730797404</v>
       </c>
-      <c r="X28" s="1" t="s">
+      <c r="X28" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="Z28" s="1" t="s">
+      <c r="Z28" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="AA28" s="1" t="s">
+      <c r="AA28" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="AB28" s="1" t="s">
+      <c r="AB28" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="AC28" s="1" t="s">
+      <c r="AC28" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="AD28" s="1" t="s">
+      <c r="AD28" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="AE28" s="1" t="s">
+      <c r="AE28" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="AF28" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG28" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH28" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI28" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ28" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK28" s="1" t="s">
+      <c r="AF28" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG28" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH28" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI28" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ28" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK28" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B29" s="1" t="s">
+      <c r="A29" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="E29" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="G29" s="1">
+      <c r="G29" s="13">
         <v>1305213723</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="13">
         <v>1410213723</v>
       </c>
-      <c r="I29" s="1" t="s">
+      <c r="I29" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="13">
         <v>10000</v>
       </c>
-      <c r="L29" s="1">
+      <c r="L29" s="14">
         <v>46054</v>
       </c>
-      <c r="N29" s="1" t="s">
+      <c r="N29" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="O29" s="1">
+      <c r="O29" s="14">
         <v>38161</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="15">
         <v>1042040244</v>
       </c>
-      <c r="Q29" s="1" t="s">
+      <c r="Q29" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="R29" s="1">
+      <c r="R29" s="15">
         <v>2311580512005</v>
       </c>
-      <c r="V29" s="1" t="s">
+      <c r="V29" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="W29" s="1">
+      <c r="W29" s="13">
         <v>1782371767</v>
       </c>
-      <c r="X29" s="1" t="s">
+      <c r="X29" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="Z29" s="1" t="s">
+      <c r="Z29" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="AA29" s="1" t="s">
+      <c r="AA29" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="AB29" s="1" t="s">
+      <c r="AB29" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="AC29" s="1" t="s">
+      <c r="AC29" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="AD29" s="1" t="s">
+      <c r="AD29" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="AE29" s="1" t="s">
+      <c r="AE29" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="AF29" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG29" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH29" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI29" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ29" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK29" s="1" t="s">
+      <c r="AF29" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG29" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH29" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI29" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ29" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK29" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B30" s="1" t="s">
+      <c r="A30" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E30" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="G30" s="1">
+      <c r="G30" s="13">
         <v>1990757830</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="13">
         <v>1410173774</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="I30" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="13">
         <v>10000</v>
       </c>
-      <c r="L30" s="1">
+      <c r="L30" s="14">
         <v>46054</v>
       </c>
-      <c r="N30" s="1" t="s">
+      <c r="N30" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="O30" s="1">
+      <c r="O30" s="14">
         <v>33970</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="15">
         <v>2824445262</v>
       </c>
-      <c r="Q30" s="1" t="s">
+      <c r="Q30" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="R30" s="1" t="s">
+      <c r="R30" s="15">
+        <v>7017344002631</v>
+      </c>
+      <c r="V30" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="V30" s="1" t="s">
+      <c r="W30" s="13">
+        <v>1925717710</v>
+      </c>
+      <c r="X30" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="W30" s="1">
-        <v>1925717710</v>
-      </c>
-      <c r="X30" s="1" t="s">
+      <c r="Z30" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA30" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="AB30" s="13" t="s">
         <v>225</v>
       </c>
-      <c r="Z30" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="AA30" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="AB30" s="1" t="s">
+      <c r="AC30" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="AC30" s="1" t="s">
+      <c r="AD30" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="AD30" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="AE30" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="AF30" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG30" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH30" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI30" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ30" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK30" s="1" t="s">
+      <c r="AE30" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="AF30" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG30" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH30" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI30" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ30" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK30" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="A31" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="D31" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="G31" s="13">
+        <v>1763122889</v>
+      </c>
+      <c r="H31" s="13">
+        <v>1410720313</v>
+      </c>
+      <c r="I31" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G31" s="1">
-        <v>1763122889</v>
-      </c>
-      <c r="H31" s="1">
-        <v>1410720313</v>
-      </c>
-      <c r="I31" s="1" t="s">
+      <c r="J31" s="13">
+        <v>10000</v>
+      </c>
+      <c r="L31" s="14">
+        <v>46143</v>
+      </c>
+      <c r="N31" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="O31" s="14">
+        <v>36906</v>
+      </c>
+      <c r="P31" s="15">
+        <v>8263476999</v>
+      </c>
+      <c r="Q31" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="R31" s="15">
+        <v>1731580441218</v>
+      </c>
+      <c r="S31" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="T31" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="J31" s="1">
-        <v>10000</v>
-      </c>
-      <c r="L31" s="1">
-        <v>46143</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="O31" s="1">
-        <v>36906</v>
-      </c>
-      <c r="P31" s="1">
-        <v>8263476999</v>
-      </c>
-      <c r="Q31" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="R31" s="1">
-        <v>1731580441218</v>
-      </c>
-      <c r="S31" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="T31" s="1" t="s">
+      <c r="U31" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="U31" s="1" t="s">
+      <c r="V31" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="V31" s="1" t="s">
+      <c r="W31" s="13">
+        <v>1325533299</v>
+      </c>
+      <c r="X31" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="Y31" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="W31" s="1">
-        <v>1325533299</v>
-      </c>
-      <c r="X31" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="Y31" s="1" t="s">
+      <c r="Z31" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="AA31" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="AB31" s="13" t="s">
         <v>235</v>
       </c>
-      <c r="Z31" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="AA31" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="AB31" s="1" t="s">
+      <c r="AC31" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="AC31" s="1" t="s">
+      <c r="AD31" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="AD31" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="AE31" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="AF31" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG31" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH31" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI31" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ31" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK31" s="1" t="s">
+      <c r="AE31" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="AF31" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG31" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH31" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI31" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ31" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK31" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B32" s="1" t="s">
+      <c r="A32" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="D32" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="E32" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="G32" s="13">
+        <v>1984397910</v>
+      </c>
+      <c r="H32" s="13">
+        <v>1410031485</v>
+      </c>
+      <c r="I32" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G32" s="1">
-        <v>1984397910</v>
-      </c>
-      <c r="H32" s="1">
-        <v>1410031485</v>
-      </c>
-      <c r="I32" s="1" t="s">
+      <c r="J32" s="13">
+        <v>10000</v>
+      </c>
+      <c r="L32" s="14">
+        <v>46143</v>
+      </c>
+      <c r="N32" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="O32" s="14">
+        <v>31902</v>
+      </c>
+      <c r="P32" s="15">
+        <v>5546839951</v>
+      </c>
+      <c r="Q32" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="R32" s="15">
+        <v>1731580504974</v>
+      </c>
+      <c r="S32" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="T32" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="U32" s="13" t="s">
         <v>241</v>
       </c>
-      <c r="J32" s="1">
-        <v>10000</v>
-      </c>
-      <c r="L32" s="1">
-        <v>46143</v>
-      </c>
-      <c r="N32" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="O32" s="1">
-        <v>31902</v>
-      </c>
-      <c r="P32" s="1">
-        <v>5546839951</v>
-      </c>
-      <c r="Q32" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="R32" s="1">
-        <v>1731580504974</v>
-      </c>
-      <c r="S32" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="T32" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="U32" s="1" t="s">
+      <c r="V32" s="13" t="s">
         <v>242</v>
       </c>
-      <c r="V32" s="1" t="s">
+      <c r="W32" s="13">
+        <v>1812206330</v>
+      </c>
+      <c r="X32" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="Y32" s="13" t="s">
         <v>243</v>
       </c>
-      <c r="W32" s="1">
-        <v>1812206330</v>
-      </c>
-      <c r="X32" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="Y32" s="1" t="s">
+      <c r="Z32" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA32" s="13" t="s">
         <v>244</v>
       </c>
-      <c r="Z32" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="AA32" s="1" t="s">
+      <c r="AB32" s="13" t="s">
         <v>245</v>
       </c>
-      <c r="AB32" s="1" t="s">
+      <c r="AC32" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="AC32" s="1" t="s">
+      <c r="AD32" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="AD32" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="AE32" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="AF32" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG32" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH32" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI32" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ32" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK32" s="1" t="s">
+      <c r="AE32" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="AF32" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG32" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH32" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI32" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ32" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK32" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B33" s="1" t="s">
+      <c r="A33" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="D33" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="E33" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="G33" s="13">
+        <v>1319047328</v>
+      </c>
+      <c r="H33" s="13">
+        <v>1410284216</v>
+      </c>
+      <c r="I33" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G33" s="1">
-        <v>1319047328</v>
-      </c>
-      <c r="H33" s="1">
-        <v>1410284216</v>
-      </c>
-      <c r="I33" s="1" t="s">
+      <c r="J33" s="13">
+        <v>10000</v>
+      </c>
+      <c r="L33" s="14">
+        <v>46153</v>
+      </c>
+      <c r="N33" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="O33" s="14">
+        <v>36835</v>
+      </c>
+      <c r="P33" s="15">
+        <v>5579571190</v>
+      </c>
+      <c r="Q33" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="R33" s="15">
+        <v>1731580505955</v>
+      </c>
+      <c r="S33" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="T33" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="U33" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="J33" s="1">
-        <v>10000</v>
-      </c>
-      <c r="L33" s="1">
-        <v>46153</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="O33" s="1">
-        <v>36835</v>
-      </c>
-      <c r="P33" s="1">
-        <v>5579571190</v>
-      </c>
-      <c r="Q33" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="R33" s="1">
-        <v>1731580505955</v>
-      </c>
-      <c r="S33" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="T33" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="U33" s="1" t="s">
+      <c r="V33" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="V33" s="1" t="s">
+      <c r="W33" s="13">
+        <v>1834674262</v>
+      </c>
+      <c r="X33" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="W33" s="1">
-        <v>1834674262</v>
-      </c>
-      <c r="X33" s="1" t="s">
+      <c r="Y33" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="Y33" s="1" t="s">
+      <c r="Z33" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA33" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="AB33" s="13" t="s">
+        <v>252</v>
+      </c>
+      <c r="AC33" s="13" t="s">
         <v>255</v>
       </c>
-      <c r="Z33" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="AA33" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="AB33" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="AC33" s="1" t="s">
+      <c r="AD33" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="AD33" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="AE33" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="AF33" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG33" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH33" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI33" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ33" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK33" s="1" t="s">
+      <c r="AE33" s="13" t="s">
+        <v>256</v>
+      </c>
+      <c r="AF33" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG33" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH33" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI33" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ33" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK33" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="13" t="s">
         <v>305</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="13" t="s">
+        <v>306</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>309</v>
+      </c>
+      <c r="G34" s="13">
+        <v>1918580928</v>
+      </c>
+      <c r="H34" s="13">
+        <v>1918580928</v>
+      </c>
+      <c r="L34" s="14">
+        <v>45972</v>
+      </c>
+      <c r="N34" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="O34" s="14">
+        <v>30051</v>
+      </c>
+      <c r="P34" s="15">
+        <v>4813347974417</v>
+      </c>
+      <c r="Q34" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="R34" s="15">
+        <v>7017017975193</v>
+      </c>
+      <c r="V34" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="W34" s="13">
+        <v>1712436301</v>
+      </c>
+      <c r="X34" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z34" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="AA34" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="AB34" s="13" t="s">
+        <v>310</v>
+      </c>
+      <c r="AC34" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="AD34" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="AE34" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="AF34" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG34" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH34" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI34" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ34" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK34" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F34" s="1">
-        <v>1409944002</v>
-      </c>
-      <c r="H34" s="1">
-        <v>1935593313</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="J34" s="1">
-        <v>10000</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="L34" s="1">
-        <v>46100</v>
-      </c>
-      <c r="N34" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="O34" s="1">
-        <v>38153</v>
-      </c>
-      <c r="P34" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="Q34" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="R34" s="1">
-        <v>2311580180685</v>
-      </c>
-      <c r="AK34" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="35" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>266</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F35" s="1">
-        <v>1915270104</v>
+        <v>1409944002</v>
       </c>
       <c r="H35" s="1">
-        <v>1935591816</v>
+        <v>1935593313</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="J35" s="1">
-        <v>7000</v>
+        <v>10000</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L35" s="1">
-        <v>45474</v>
-      </c>
+        <v>46100</v>
+      </c>
+      <c r="M35" s="2"/>
       <c r="N35" s="1" t="s">
         <v>157</v>
       </c>
       <c r="O35" s="1">
-        <v>38443</v>
+        <v>38153</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="Q35" s="1" t="s">
         <v>60</v>
       </c>
       <c r="R35" s="1">
-        <v>2311580121330</v>
+        <v>2311580180685</v>
       </c>
       <c r="AK35" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F36" s="1">
-        <v>1915270105</v>
+        <v>1915270104</v>
       </c>
       <c r="H36" s="1">
-        <v>1935591916</v>
+        <v>1935591816</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="J36" s="1">
-        <v>9500</v>
+        <v>7000</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L36" s="1">
-        <v>45909</v>
-      </c>
+        <v>45474</v>
+      </c>
+      <c r="M36" s="2"/>
       <c r="N36" s="1" t="s">
         <v>157</v>
       </c>
       <c r="O36" s="1">
-        <v>38952</v>
+        <v>38443</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="Q36" s="1" t="s">
         <v>60</v>
       </c>
       <c r="R36" s="1">
-        <v>2311580453888</v>
+        <v>2311580121330</v>
       </c>
       <c r="AK36" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F37" s="1">
-        <v>1967042950</v>
+        <v>1915270105</v>
       </c>
       <c r="H37" s="1">
-        <v>1935592484</v>
+        <v>1935591916</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="J37" s="1">
         <v>9500</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L37" s="1">
         <v>45909</v>
       </c>
+      <c r="M37" s="2"/>
       <c r="N37" s="1" t="s">
         <v>157</v>
       </c>
       <c r="O37" s="1">
-        <v>38688</v>
+        <v>38952</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="Q37" s="1" t="s">
         <v>60</v>
       </c>
       <c r="R37" s="1">
-        <v>2311030382527</v>
+        <v>2311580453888</v>
       </c>
       <c r="AK37" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="38" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F38" s="1">
-        <v>1986686877</v>
+        <v>1967042950</v>
       </c>
       <c r="H38" s="1">
-        <v>1935591836</v>
+        <v>1935592484</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="J38" s="1">
-        <v>7000</v>
+        <v>9500</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L38" s="1">
-        <v>45658</v>
-      </c>
+        <v>45909</v>
+      </c>
+      <c r="M38" s="2"/>
       <c r="N38" s="1" t="s">
         <v>157</v>
       </c>
       <c r="O38" s="1">
-        <v>37483</v>
+        <v>38688</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="Q38" s="1" t="s">
         <v>60</v>
       </c>
       <c r="R38" s="1">
-        <v>2311580181156</v>
+        <v>2311030382527</v>
       </c>
       <c r="AK38" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="39" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F39" s="1">
-        <v>1986686878</v>
+        <v>1986686877</v>
       </c>
       <c r="H39" s="1">
-        <v>1935591828</v>
+        <v>1935591836</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="J39" s="1">
-        <v>10500</v>
+        <v>7000</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L39" s="1">
-        <v>46027</v>
-      </c>
+        <v>45658</v>
+      </c>
+      <c r="M39" s="2"/>
       <c r="N39" s="1" t="s">
         <v>157</v>
       </c>
       <c r="O39" s="1">
-        <v>35286</v>
+        <v>37483</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="Q39" s="1" t="s">
         <v>60</v>
       </c>
       <c r="R39" s="1">
-        <v>1731030011244</v>
+        <v>2311580181156</v>
       </c>
       <c r="AK39" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="40" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F40" s="1">
-        <v>1986686879</v>
+        <v>1986686878</v>
       </c>
       <c r="H40" s="1">
-        <v>1935592119</v>
+        <v>1935591828</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="J40" s="1">
-        <v>7500</v>
+        <v>10500</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L40" s="1">
-        <v>45292</v>
-      </c>
+        <v>46027</v>
+      </c>
+      <c r="M40" s="2"/>
       <c r="N40" s="1" t="s">
         <v>157</v>
       </c>
       <c r="O40" s="1">
-        <v>37244</v>
+        <v>35286</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="Q40" s="1" t="s">
         <v>60</v>
       </c>
       <c r="R40" s="1">
-        <v>2311580116900</v>
+        <v>1731030011244</v>
       </c>
       <c r="AK40" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="41" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="G41" s="1">
-        <v>1611169592</v>
+        <v>58</v>
+      </c>
+      <c r="F41" s="1">
+        <v>1986686879</v>
       </c>
       <c r="H41" s="1">
-        <v>1999968844</v>
+        <v>1935592119</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>298</v>
+        <v>291</v>
+      </c>
+      <c r="J41" s="1">
+        <v>7500</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>261</v>
       </c>
       <c r="L41" s="1">
-        <v>45931</v>
+        <v>45292</v>
+      </c>
+      <c r="M41" s="2"/>
+      <c r="N41" s="1" t="s">
+        <v>157</v>
       </c>
       <c r="O41" s="1">
-        <v>31821</v>
+        <v>37244</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="Q41" s="1" t="s">
         <v>60</v>
       </c>
       <c r="R41" s="1">
-        <v>2311580467330</v>
+        <v>2311580116900</v>
       </c>
       <c r="AK41" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="G42" s="1">
+        <v>1611169592</v>
+      </c>
+      <c r="H42" s="1">
+        <v>1999968844</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="L42" s="1">
+        <v>45931</v>
+      </c>
+      <c r="M42" s="2"/>
+      <c r="O42" s="1">
+        <v>31821</v>
+      </c>
+      <c r="P42" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="Q42" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="R42" s="1">
+        <v>2311580467330</v>
+      </c>
+      <c r="AK42" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="E43" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="H43" s="1">
+        <v>1935600928</v>
+      </c>
+      <c r="I43" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="E42" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="H42" s="1">
-        <v>1935600928</v>
-      </c>
-      <c r="I42" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="AK42" s="1" t="s">
+      <c r="M43" s="2"/>
+      <c r="AK43" s="1" t="s">
         <v>81</v>
       </c>
     </row>

</xml_diff>